<commit_message>
final test plan in xlsx format
</commit_message>
<xml_diff>
--- a/test plan.xlsx
+++ b/test plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\projects\playwright_redmine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BCE0180-0805-42AB-A7F7-BFD34CE3C507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4876983-7EDE-423D-BCE7-9ACE5E7BA800}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="77">
   <si>
     <t>TEST PLAN</t>
   </si>
@@ -66,9 +66,6 @@
     <t>h2 "Features" is visible</t>
   </si>
   <si>
-    <t>Find "Flexible issue tracking system" link</t>
-  </si>
-  <si>
     <t>"issue tracking system" link is visible</t>
   </si>
   <si>
@@ -90,9 +87,6 @@
     <t>Find label "Search" with inner &lt;a&gt; link and click</t>
   </si>
   <si>
-    <t>Check search form accessability</t>
-  </si>
-  <si>
     <t>form#search-form is visible</t>
   </si>
   <si>
@@ -105,16 +99,10 @@
     <t>Click on check-box with id "titles_only"</t>
   </si>
   <si>
-    <t>Attribute "checked" values must be "checked"</t>
-  </si>
-  <si>
     <t>Find input with id "search-input"</t>
   </si>
   <si>
     <t>input with id "search-input" must be visible</t>
-  </si>
-  <si>
-    <t>Enter invalid text "sqs"</t>
   </si>
   <si>
     <t>The entered data is shown in
@@ -124,9 +112,6 @@
     <t>Click on input with type "submit"</t>
   </si>
   <si>
-    <t>Results are 0</t>
-  </si>
-  <si>
     <t>Enter valid text "error"</t>
   </si>
   <si>
@@ -134,13 +119,154 @@
   </si>
   <si>
     <t>but it does not, because site is static</t>
+  </si>
+  <si>
+    <t>C03</t>
+  </si>
+  <si>
+    <t>Edit task in roadmap (negative)</t>
+  </si>
+  <si>
+    <t>Find label "Roadmap" in menu and click</t>
+  </si>
+  <si>
+    <t>User is not logged in</t>
+  </si>
+  <si>
+    <t>C04</t>
+  </si>
+  <si>
+    <t>Find label "Issues" in menu and click</t>
+  </si>
+  <si>
+    <t>Issue filter by category on issue page</t>
+  </si>
+  <si>
+    <t>Find "Flexible issue tracking system" link-text</t>
+  </si>
+  <si>
+    <t>Check search form visual accessability</t>
+  </si>
+  <si>
+    <t>Attribute "checked" value must be "checked"</t>
+  </si>
+  <si>
+    <t>Scroll and find article with header "7.0.1"</t>
+  </si>
+  <si>
+    <t>Article with header "7.0.1" is visible</t>
+  </si>
+  <si>
+    <t>Find first issue in the article table</t>
+  </si>
+  <si>
+    <t>First row issue is visible</t>
+  </si>
+  <si>
+    <t>Find options for this issue</t>
+  </si>
+  <si>
+    <t>Options for this issue is visible</t>
+  </si>
+  <si>
+    <t>Click on options button</t>
+  </si>
+  <si>
+    <t>Opened tab (unordered list) with actions</t>
+  </si>
+  <si>
+    <t>Find and click 'delete' option</t>
+  </si>
+  <si>
+    <t>Nothing happens because button disabled. Row with current issue still exists in table</t>
+  </si>
+  <si>
+    <t>Instead of cookies, on website redmine.org it can be error with heavy load. It must be catched and make page reloading.</t>
+  </si>
+  <si>
+    <t>Find filter by status of issue</t>
+  </si>
+  <si>
+    <t>Selectbox for status is visible</t>
+  </si>
+  <si>
+    <t>Click on it and find closed option</t>
+  </si>
+  <si>
+    <t>Saved option in box</t>
+  </si>
+  <si>
+    <t>Find submit button and click on it</t>
+  </si>
+  <si>
+    <t>Closed issue status is correct in table of issues and on their pages</t>
+  </si>
+  <si>
+    <t>Must be in table only issues with closed status</t>
+  </si>
+  <si>
+    <t>Find first row id and click</t>
+  </si>
+  <si>
+    <t>Must open page with id in url and in header</t>
+  </si>
+  <si>
+    <t>Find badge "closed"</t>
+  </si>
+  <si>
+    <t>Must be visible badge "closed"</t>
+  </si>
+  <si>
+    <t>C05</t>
+  </si>
+  <si>
+    <t>Find "Add filter" button and click</t>
+  </si>
+  <si>
+    <t>Opened select-tab with options</t>
+  </si>
+  <si>
+    <t>Find "Category" option and click</t>
+  </si>
+  <si>
+    <t>Must be visible row-filter "Category"</t>
+  </si>
+  <si>
+    <t>Find filter with id "operators_category_id" and click</t>
+  </si>
+  <si>
+    <t>Find option with value="=" and click</t>
+  </si>
+  <si>
+    <t>Selected option with value "="</t>
+  </si>
+  <si>
+    <t>Find filter with id "values_category_id_1" and click</t>
+  </si>
+  <si>
+    <t>Find "Feeds" option and click</t>
+  </si>
+  <si>
+    <t>Selected option with value "18" and text Feeds</t>
+  </si>
+  <si>
+    <t>Must be in table only issues with Category "Feeds"</t>
+  </si>
+  <si>
+    <t>Find Category div and check value of it</t>
+  </si>
+  <si>
+    <t>Must be "Category: Feeds"</t>
+  </si>
+  <si>
+    <t>Tests cover only desktop browser version with FullHD resolution</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -166,6 +292,14 @@
     <font>
       <b/>
       <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -199,11 +333,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -214,6 +345,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -496,256 +642,705 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D24"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D70"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" style="2"/>
-    <col min="2" max="2" width="42.453125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="51.36328125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="19.1796875" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="2"/>
+    <col min="1" max="1" width="8.7109375" style="1"/>
+    <col min="2" max="2" width="42.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="51.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="22.5703125" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="3" spans="1:4" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+    </row>
+    <row r="2" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+    </row>
+    <row r="3" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-    </row>
-    <row r="4" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>1</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>2</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>3</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-    </row>
-    <row r="5" spans="1:4" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+      <c r="B14" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B15" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>1</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>2</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D18" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="26.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
         <v>1</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="2">
+      <c r="B19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
         <v>2</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="44.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2">
+      <c r="B20" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
         <v>3</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
+      <c r="B21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>4</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>5</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>6</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B27" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-    </row>
-    <row r="13" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B29" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="2">
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="4">
         <v>1</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B30" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="2">
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="4">
         <v>2</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
+      <c r="B31" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>3</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B33" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C33" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D33" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="2">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="4">
         <v>1</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="2">
+      <c r="B34" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="4">
         <v>2</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="2">
+      <c r="B35" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="4">
         <v>3</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D19" s="2" t="s">
+      <c r="B36" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="4">
+        <v>4</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A38" s="4">
+        <v>5</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C41" s="7"/>
+      <c r="D41" s="7"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="4" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="2">
+      <c r="B42" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="A21" s="2">
+      <c r="B43" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="2">
+      <c r="C43" s="7"/>
+      <c r="D43" s="7"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="4">
+        <v>1</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C44" s="6"/>
+      <c r="D44" s="6"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="4">
+        <v>2</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C45" s="6"/>
+      <c r="D45" s="6"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="4">
+        <v>3</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C46" s="6"/>
+      <c r="D46" s="6"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B47" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="A23" s="2">
+      <c r="C47" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="A24" s="2">
+      <c r="D47" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C24" s="2" t="s">
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="4">
+        <v>1</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D48" s="4"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="4">
+        <v>2</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D49" s="4"/>
+    </row>
+    <row r="50" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="5">
+        <v>3</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="5">
+        <v>4</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="5">
+        <v>5</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C55" s="7"/>
+      <c r="D55" s="7"/>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C56" s="6"/>
+      <c r="D56" s="6"/>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C57" s="7"/>
+      <c r="D57" s="7"/>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="4">
+        <v>1</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C58" s="6"/>
+      <c r="D58" s="6"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="4">
+        <v>2</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C59" s="6"/>
+      <c r="D59" s="6"/>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="4">
+        <v>3</v>
+      </c>
+      <c r="B60" s="6" t="s">
         <v>33</v>
       </c>
+      <c r="C60" s="6"/>
+      <c r="D60" s="6"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="4">
+        <v>1</v>
+      </c>
+      <c r="B62" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D62" s="4"/>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="4">
+        <v>2</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D63" s="4"/>
+    </row>
+    <row r="64" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>3</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
+        <v>4</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A66" s="1">
+        <v>5</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>6</v>
+      </c>
+      <c r="B67" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C67" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>7</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" s="1">
+        <v>8</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
+        <v>9</v>
+      </c>
+      <c r="B70" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>75</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="B12:D12"/>
+  <mergeCells count="28">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B6:D6"/>
     <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B28:D28"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="B59:D59"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>